<commit_message>
Refactor transport input types and codes
Correction d'erreurs, il y avait un système avec un binding sur un CodeSystem 0b5512e00bf4400da1c332991883b1ee98b3d51b
</commit_message>
<xml_diff>
--- a/nriss-patch-2/ig/StructureDefinition-fr-diagnostic-report-imaging-document.xlsx
+++ b/nriss-patch-2/ig/StructureDefinition-fr-diagnostic-report-imaging-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-27T15:58:47+00:00</t>
+    <t>2026-08-04T07:44:41+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -609,7 +609,7 @@
     <t>serviceRequestAccessionNumber</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-service-request-document|0.1.0)
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-service-request-imaging-document|0.1.0)
 </t>
   </si>
   <si>

</xml_diff>